<commit_message>
Q30 production kiln; green highlight on edited cells
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -82,8 +82,25 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF006100"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -130,6 +147,11 @@
         <fgColor rgb="FFF5F8FC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -158,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -209,6 +231,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -592,6 +621,11 @@
           <t xml:space="preserve">Общий тест ОПП — 30 вопросов </t>
         </is>
       </c>
+      <c r="K1" s="24" t="inlineStr">
+        <is>
+          <t>Зелёным выделены исправленные (ранее жёлтые/красные) ячейки</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="n"/>
@@ -657,7 +691,7 @@
           <t>Максимального наращивания выпуска экспортных поддонов при полном исключении студентов из производственного контура</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Проведения только лекционного курса по Индустрии 4.0 без работы студентов на действующей линии                    </t>
         </is>
@@ -1027,12 +1061,12 @@
           <t>Экономика производства как дисциплина в первую очередь изучает:</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Биржевые котировки и курсы валют без связи с превращением ресурсов цеха в готовую продукцию        </t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Только методы ценообразования ритейла без анализа материальных и трудовых затрат производства      </t>
         </is>
@@ -1042,7 +1076,7 @@
           <t>Экономические отношения в процессе превращения материальных и трудовых ресурсов в готовую продукцию</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F14" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Только налоговые режимы региона без рассмотрения преобразования ресурсов в изделие предприятия     </t>
         </is>
@@ -1065,7 +1099,7 @@
           <t>В модуле по экономике производства выделены четыре смысловых блока. Какой набор верный?</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Маркетинг бренда, розничная сеть, упаковка товара и работа call-центра без учёта себестоимости   </t>
         </is>
@@ -1075,12 +1109,12 @@
           <t xml:space="preserve">Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства   </t>
         </is>
       </c>
-      <c r="E15" s="23" t="inlineStr">
+      <c r="E15" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Кредитная политика банка, валютный контроль, страхование грузов и таможенное оформление поставок </t>
         </is>
       </c>
-      <c r="F15" s="23" t="inlineStr">
+      <c r="F15" s="25" t="inlineStr">
         <is>
           <t>Корпоративная культура, соцпакет, охрана труда и мотивация персонала без финансовых блоков модуля</t>
         </is>
@@ -1103,12 +1137,12 @@
           <t>Базовый комплект финансовой отчётности предприятия обычно включает:</t>
         </is>
       </c>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="C16" s="25" t="inlineStr">
         <is>
           <t>Только ведомость амортизации станков и карточки инвентарных объектов без полного комплекта отчётности</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D16" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Только декларация по НДС и выписка расчётного счёта без баланса, прибылей и движения денег           </t>
         </is>
@@ -1118,7 +1152,7 @@
           <t xml:space="preserve">Отчёт о прибылях и убытках, бухгалтерский баланс и отчёт о движении денежных средств за период       </t>
         </is>
       </c>
-      <c r="F16" s="20" t="inlineStr">
+      <c r="F16" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Только прогноз продаж маркетинга и план рекламного бюджета без основных форм финансовой отчётности   </t>
         </is>
@@ -1141,17 +1175,17 @@
           <t>Себестоимость единицы продукции — это:</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Рыночная цена, которую выставил отдел продаж без калькуляции собственных затрат предприятия        </t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Только прямые затраты на пиломатериал без включения труда, энергии, амортизации и сбыта изделия    </t>
         </is>
       </c>
-      <c r="E17" s="23" t="inlineStr">
+      <c r="E17" s="25" t="inlineStr">
         <is>
           <t>Плановая выручка партии, механически делённая на число рабочих смены, без полной калькуляции затрат</t>
         </is>
@@ -1179,7 +1213,7 @@
           <t>Себестоимость напрямую влияет на три управленческих показателя. Какие?</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="C18" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Только численность административного персонала без выхода на цену, конкуренцию и прибыль         </t>
         </is>
@@ -1189,12 +1223,12 @@
           <t xml:space="preserve">Цену предложения на рынке, конкурентоспособность продукции и итоговую прибыльность бизнеса       </t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Только график плановых ремонтов линии без влияния на предложение рынку и прибыльность бизнеса    </t>
         </is>
       </c>
-      <c r="F18" s="20" t="inlineStr">
+      <c r="F18" s="25" t="inlineStr">
         <is>
           <t>Только внутренний индекс текучести кадров без связи с ценой изделия и итоговой маржой предприятия</t>
         </is>
@@ -1217,12 +1251,12 @@
           <t>Бюджет на предприятии — это прежде всего:</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C19" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Фактический отчёт кассы за прошедшие сутки без утверждённых плановых лимитов на период      </t>
         </is>
       </c>
-      <c r="D19" s="23" t="inlineStr">
+      <c r="D19" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Реестр уже оплаченных счетов поставщиков без заранее заданных доходов и расходов периода    </t>
         </is>
@@ -1232,7 +1266,7 @@
           <t>Плановый документ доходов и расходов на выбранный период: месяц, квартал или календарный год</t>
         </is>
       </c>
-      <c r="F19" s="23" t="inlineStr">
+      <c r="F19" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Журнал закрытых бухгалтерских проводок месяца без плановых назначений доходов и расходов    </t>
         </is>
@@ -1255,17 +1289,17 @@
           <t>Под масштабированием в контексте производства понимают:</t>
         </is>
       </c>
-      <c r="C20" s="20" t="inlineStr">
+      <c r="C20" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Сокращение ассортимента до одной позиции без роста выпуска, доли рынка и снижения удельных издержек </t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D20" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Заморозка инвестиций и консервация части мощностей ради снижения, а не роста объёма выпуска         </t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E20" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Увеличение только офисного штата управляющей компании без расширения выпуска и снижения издержек    </t>
         </is>
@@ -1298,17 +1332,17 @@
           <t>Рост «вглубь» цепочки стоимости — контроль поставок сырья и/или выход ближе к конечному потребителю</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Горизонтальный рост числа однотипных линий того же передела без входа в сырьё и к потребителю      </t>
         </is>
       </c>
-      <c r="E21" s="23" t="inlineStr">
+      <c r="E21" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Концентрический выпуск непрофильных изделий под брендом без контроля поставок и каналов сбыта      </t>
         </is>
       </c>
-      <c r="F21" s="23" t="inlineStr">
+      <c r="F21" s="25" t="inlineStr">
         <is>
           <t>Организационное увеличение штата администрации без изменения цепочки стоимости и близости к клиенту</t>
         </is>
@@ -1331,12 +1365,12 @@
           <t>Инвестиции в производство — это:</t>
         </is>
       </c>
-      <c r="C22" s="20" t="inlineStr">
+      <c r="C22" s="25" t="inlineStr">
         <is>
           <t>Текущие платежи за энергию и расходники без прироста мощностей, качества и конкурентоспособности</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D22" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Компенсация брака прошлых периодов без плана роста выпуска, качества продукции и доли рынка     </t>
         </is>
@@ -1346,7 +1380,7 @@
           <t xml:space="preserve">Вложения капитала с целью роста объёма выпуска, качества продукции и конкурентоспособности      </t>
         </is>
       </c>
-      <c r="F22" s="20" t="inlineStr">
+      <c r="F22" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Возврат ранее взятого кредита без создания новых мощностей и улучшения конкурентоспособности    </t>
         </is>
@@ -1369,7 +1403,7 @@
           <t>Какие четыре вида инвестиций названы в учебном модуле?</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Прямые, косвенные, накладные и коммерческие затраты в калькуляции единицы готовой продукции </t>
         </is>
@@ -1379,12 +1413,12 @@
           <t xml:space="preserve">Капитальные, инновационные, операционные и финансовые вложения в развитие предприятия       </t>
         </is>
       </c>
-      <c r="E23" s="23" t="inlineStr">
+      <c r="E23" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Краткосрочные, среднесрочные, долгосрочные и бессрочные обязательства в структуре баланса   </t>
         </is>
       </c>
-      <c r="F23" s="23" t="inlineStr">
+      <c r="F23" s="25" t="inlineStr">
         <is>
           <t>Постоянные, переменные, смешанные и маржинальные издержки в управленческом учёте предприятия</t>
         </is>
@@ -1407,17 +1441,17 @@
           <t>В чём принципиальная разница цифровизации и автоматизации?</t>
         </is>
       </c>
-      <c r="C24" s="20" t="inlineStr">
+      <c r="C24" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Цифровизация заменяет людей машинами, а автоматизация лишь хранит сканы бумажных документов           </t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D24" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Автоматизация переводит процессы в данные, а цифровизация сводится к закупке дополнительных датчиков  </t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E24" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Оба термина означают только установку серверов без изменения цеховых и управленческих процессов       </t>
         </is>
@@ -1673,17 +1707,17 @@
           <t>ТСД в контуре WMS — это:</t>
         </is>
       </c>
-      <c r="C31" s="23" t="inlineStr">
+      <c r="C31" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Стационарный сервер WMS, на котором хранятся складские справочники, остатки и история движений           </t>
         </is>
       </c>
-      <c r="D31" s="23" t="inlineStr">
+      <c r="D31" s="25" t="inlineStr">
         <is>
           <t>Принтер этикеток на воротах приёмки, который только печатает коды, но сам складские операции не сканирует</t>
         </is>
       </c>
-      <c r="E31" s="23" t="inlineStr">
+      <c r="E31" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Модуль расчёта зарплаты кладовщиков в ERP без функций сканирования штрих- и QR-кодов на складе           </t>
         </is>
@@ -1711,7 +1745,7 @@
           <t>Какой набор мер соответствует защите промышленного IT-контура в модуле?</t>
         </is>
       </c>
-      <c r="C32" s="20" t="inlineStr">
+      <c r="C32" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Открытый удалённый доступ ко всем контроллерам линии без пароля ради удобства дежурной смены          </t>
         </is>
@@ -1721,12 +1755,12 @@
           <t>Мониторинг сетевого трафика, межсетевые экраны и антивирусы, резервное копирование, обучение персонала</t>
         </is>
       </c>
-      <c r="E32" s="20" t="inlineStr">
+      <c r="E32" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Хранение единственной копии SCADA на диске оператора без резервирования и контроля сетевого периметра </t>
         </is>
       </c>
-      <c r="F32" s="20" t="inlineStr">
+      <c r="F32" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Общая учётная запись «оператор» во всех системах без разграничения прав, экранов и резервных копий    </t>
         </is>
@@ -1744,37 +1778,37 @@
       <c r="A33" s="22" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="23" t="inlineStr">
-        <is>
-          <t>Почему компрометация ERP опасна для всего предприятия, а не только для IT-службы?</t>
-        </is>
-      </c>
-      <c r="C33" s="23" t="inlineStr">
-        <is>
-          <t>Через ERP связаны производство, склад, продажи и финансы, поэтому сбой сразу бьёт по заказам и отгрузке</t>
-        </is>
-      </c>
-      <c r="D33" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Потому что ERP хранит лишь архив презентаций для инвесторов и не участвует в операционном контуре      </t>
-        </is>
-      </c>
-      <c r="E33" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Потому что потеря ERP затрагивает только оформление визиток и не останавливает склад и отгрузку        </t>
-        </is>
-      </c>
-      <c r="F33" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Потому что ERP изолирована от склада и продаж и используется исключительно службой маркетинга          </t>
-        </is>
-      </c>
-      <c r="G33" s="21" t="n">
+      <c r="B33" s="25" t="inlineStr">
+        <is>
+          <t>Почему пиломатериал перед сборкой каркаса поддона пропускают через сушильную камеру?</t>
+        </is>
+      </c>
+      <c r="C33" s="25" t="inlineStr">
+        <is>
+          <t>Чтобы стабилизировать геометрию досок, снизить риск трещин, плесени и ослабления крепежа в эксплуатации</t>
+        </is>
+      </c>
+      <c r="D33" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Чтобы сырые доски стали тяжелее и промышленный манипулятор надёжнее удерживал заготовку в захвате      </t>
+        </is>
+      </c>
+      <c r="E33" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Чтобы клеймо ISPM-15 само проявилось на влажной поверхности без отдельной маркировочной станции        </t>
+        </is>
+      </c>
+      <c r="F33" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Чтобы конвейер сборки работал медленнее и такт роботизированной ячейки искусственно удлинился          </t>
+        </is>
+      </c>
+      <c r="G33" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="H33" s="23" t="inlineStr">
-        <is>
-          <t>Через ERP связаны производство, склад, продажи и финансы, поэтому сбой сразу бьёт по заказам и отгрузке</t>
+      <c r="H33" s="25" t="inlineStr">
+        <is>
+          <t>Чтобы стабилизировать геометрию досок, снизить риск трещин, плесени и ослабления крепежа в эксплуатации</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify rewritten answers, keep green highlight
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="K1" s="24" t="inlineStr">
         <is>
-          <t>Зелёным выделены исправленные (ранее жёлтые/красные) ячейки</t>
+          <t>Зелёным — исправленные ответы (проще, без научных терминов)</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="E4" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Проведения только лекционного курса по Индустрии 4.0 без работы студентов на действующей линии                    </t>
+          <t xml:space="preserve">Проведения только лекций про умный завод без работы студентов на настоящей линии                                  </t>
         </is>
       </c>
       <c r="F4" s="20" t="inlineStr">
@@ -1063,12 +1063,12 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Биржевые котировки и курсы валют без связи с превращением ресурсов цеха в готовую продукцию        </t>
+          <t xml:space="preserve">Как меняются цены акций на бирже, без связи с тем, как в цехе из досок делают поддон               </t>
         </is>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Только методы ценообразования ритейла без анализа материальных и трудовых затрат производства      </t>
+          <t xml:space="preserve">Как магазины ставят ценники, без учёта сколько реально стоят доски, работа и электричество         </t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Только налоговые режимы региона без рассмотрения преобразования ресурсов в изделие предприятия     </t>
+          <t xml:space="preserve">Какие налоги платит регион, без разбора как материалы и труд превращаются в готовый поддон         </t>
         </is>
       </c>
       <c r="G14" s="21" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Маркетинг бренда, розничная сеть, упаковка товара и работа call-центра без учёта себестоимости   </t>
+          <t xml:space="preserve">Реклама, магазины, красивая коробка и телефон горячей линии — без учёта денег и себестоимости    </t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
@@ -1111,12 +1111,12 @@
       </c>
       <c r="E15" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Кредитная политика банка, валютный контроль, страхование грузов и таможенное оформление поставок </t>
+          <t xml:space="preserve">Кредиты банка, курс валюты, страховка груза и таможня — это не те четыре блока из модуля         </t>
         </is>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>Корпоративная культура, соцпакет, охрана труда и мотивация персонала без финансовых блоков модуля</t>
+          <t xml:space="preserve">Корпоративы, льготы, каски и премии сотрудникам — без финансового учёта и себестоимости          </t>
         </is>
       </c>
       <c r="G15" s="21" t="n">
@@ -1139,12 +1139,12 @@
       </c>
       <c r="C16" s="25" t="inlineStr">
         <is>
-          <t>Только ведомость амортизации станков и карточки инвентарных объектов без полного комплекта отчётности</t>
+          <t xml:space="preserve">Только список станков и сколько они износились — без прибыли, баланса и движения денег               </t>
         </is>
       </c>
       <c r="D16" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Только декларация по НДС и выписка расчётного счёта без баланса, прибылей и движения денег           </t>
+          <t xml:space="preserve">Только налоговая бумага и выписка из банка — без полного набора главных финансовых отчётов           </t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Только прогноз продаж маркетинга и план рекламного бюджета без основных форм финансовой отчётности   </t>
+          <t xml:space="preserve">Только план продаж и рекламный бюджет — без отчёта о прибыли, баланса и движения денег               </t>
         </is>
       </c>
       <c r="G16" s="21" t="n">
@@ -1177,17 +1177,17 @@
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рыночная цена, которую выставил отдел продаж без калькуляции собственных затрат предприятия        </t>
+          <t xml:space="preserve">Цена, которую продавец взял «с потолка», не считая свои реальные расходы на поддон                 </t>
         </is>
       </c>
       <c r="D17" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Только прямые затраты на пиломатериал без включения труда, энергии, амортизации и сбыта изделия    </t>
+          <t xml:space="preserve">Только цена досок, без зарплаты, электричества, износа станков и доставки покупателю               </t>
         </is>
       </c>
       <c r="E17" s="25" t="inlineStr">
         <is>
-          <t>Плановая выручка партии, механически делённая на число рабочих смены, без полной калькуляции затрат</t>
+          <t xml:space="preserve">Выручка за партию, просто делённая на число людей в смене, без подсчёта всех затрат                </t>
         </is>
       </c>
       <c r="F17" s="23" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C18" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Только численность административного персонала без выхода на цену, конкуренцию и прибыль         </t>
+          <t xml:space="preserve">Только сколько чиновников в офисе, без цены поддона, конкурентов и прибыли завода                </t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -1225,12 +1225,12 @@
       </c>
       <c r="E18" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Только график плановых ремонтов линии без влияния на предложение рынку и прибыльность бизнеса    </t>
+          <t xml:space="preserve">Только график ремонта линии, без влияния на цену, конкуренцию и прибыль                          </t>
         </is>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>Только внутренний индекс текучести кадров без связи с ценой изделия и итоговой маржой предприятия</t>
+          <t xml:space="preserve">Только как часто люди увольняются, без связи с ценой поддона и прибылью завода                   </t>
         </is>
       </c>
       <c r="G18" s="21" t="n">
@@ -1253,12 +1253,12 @@
       </c>
       <c r="C19" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Фактический отчёт кассы за прошедшие сутки без утверждённых плановых лимитов на период      </t>
+          <t xml:space="preserve">Сколько денег уже прошло через кассу вчера, без плана на месяц, квартал или год             </t>
         </is>
       </c>
       <c r="D19" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Реестр уже оплаченных счетов поставщиков без заранее заданных доходов и расходов периода    </t>
+          <t xml:space="preserve">Список уже оплаченных счетов поставщикам, без плана доходов и расходов на период            </t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Журнал закрытых бухгалтерских проводок месяца без плановых назначений доходов и расходов    </t>
+          <t xml:space="preserve">Журнал уже сделанных проводок за месяц, без заранее утверждённого плана трат и доходов      </t>
         </is>
       </c>
       <c r="G19" s="21" t="n">
@@ -1291,17 +1291,17 @@
       </c>
       <c r="C20" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сокращение ассортимента до одной позиции без роста выпуска, доли рынка и снижения удельных издержек </t>
+          <t xml:space="preserve">Оставить в продаже только один вид поддона, не увеличивая выпуск и не снижая затраты на штуку       </t>
         </is>
       </c>
       <c r="D20" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заморозка инвестиций и консервация части мощностей ради снижения, а не роста объёма выпуска         </t>
+          <t xml:space="preserve">Заморозить вложения и часть цеха остановить, чтобы выпускать меньше, а не больше                    </t>
         </is>
       </c>
       <c r="E20" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Увеличение только офисного штата управляющей компании без расширения выпуска и снижения издержек    </t>
+          <t xml:space="preserve">Набрать только офисных сотрудников, не увеличивая выпуск поддонов и не снижая затраты на штуку      </t>
         </is>
       </c>
       <c r="F20" s="20" t="inlineStr">
@@ -1334,17 +1334,17 @@
       </c>
       <c r="D21" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Горизонтальный рост числа однотипных линий того же передела без входа в сырьё и к потребителю      </t>
+          <t xml:space="preserve">Поставить рядом ещё такие же линии сборки, не заходя в сырьё и не ближе к покупателю               </t>
         </is>
       </c>
       <c r="E21" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Концентрический выпуск непрофильных изделий под брендом без контроля поставок и каналов сбыта      </t>
+          <t xml:space="preserve">Начать выпускать совсем другие товары под тем же названием, не контролируя доски и сбыт            </t>
         </is>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>Организационное увеличение штата администрации без изменения цепочки стоимости и близости к клиенту</t>
+          <t xml:space="preserve">Просто увеличить штат офиса, не меняя, кто поставляет доски и кто покупает поддоны                 </t>
         </is>
       </c>
       <c r="G21" s="21" t="n">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="C22" s="25" t="inlineStr">
         <is>
-          <t>Текущие платежи за энергию и расходники без прироста мощностей, качества и конкурентоспособности</t>
+          <t xml:space="preserve">Обычные счета за свет и расходники, от которых цех не становится больше и поддон не лучше       </t>
         </is>
       </c>
       <c r="D22" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Компенсация брака прошлых периодов без плана роста выпуска, качества продукции и доли рынка     </t>
+          <t xml:space="preserve">Оплата старого брака, без плана делать больше, качественнее и конкурентоспособнее               </t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Возврат ранее взятого кредита без создания новых мощностей и улучшения конкурентоспособности    </t>
+          <t xml:space="preserve">Возврат старого кредита банку, без новых станков и без улучшения поддона                        </t>
         </is>
       </c>
       <c r="G22" s="21" t="n">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="C23" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Прямые, косвенные, накладные и коммерческие затраты в калькуляции единицы готовой продукции </t>
+          <t xml:space="preserve">Прямые, косвенные, накладные и торговые затраты в расчёте цены одного поддона               </t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
@@ -1415,12 +1415,12 @@
       </c>
       <c r="E23" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Краткосрочные, среднесрочные, долгосрочные и бессрочные обязательства в структуре баланса   </t>
+          <t xml:space="preserve">Долги на месяц, на год, на много лет и без срока — это про долги, а не про виды вложений    </t>
         </is>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>Постоянные, переменные, смешанные и маржинальные издержки в управленческом учёте предприятия</t>
+          <t xml:space="preserve">Затраты постоянные, переменные и смешанные — это про расходы, а не про четыре вида вложений </t>
         </is>
       </c>
       <c r="G23" s="21" t="n">
@@ -1443,17 +1443,17 @@
       </c>
       <c r="C24" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Цифровизация заменяет людей машинами, а автоматизация лишь хранит сканы бумажных документов           </t>
+          <t xml:space="preserve">Цифровизация якобы ставит роботов вместо людей, а автоматизация только сканирует бумажки              </t>
         </is>
       </c>
       <c r="D24" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Автоматизация переводит процессы в данные, а цифровизация сводится к закупке дополнительных датчиков  </t>
+          <t xml:space="preserve">Автоматизация якобы переводит всё в цифру, а цифровизация — это просто купить ещё датчики             </t>
         </is>
       </c>
       <c r="E24" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Оба термина означают только установку серверов без изменения цеховых и управленческих процессов       </t>
+          <t xml:space="preserve">Оба слова якобы значат только «купили сервер», без изменений в цехе и в управлении                    </t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
@@ -1709,17 +1709,17 @@
       </c>
       <c r="C31" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Стационарный сервер WMS, на котором хранятся складские справочники, остатки и история движений           </t>
+          <t xml:space="preserve">Большой компьютер склада, где лежат списки товара и остатки, но им не сканируют коробки в руках          </t>
         </is>
       </c>
       <c r="D31" s="25" t="inlineStr">
         <is>
-          <t>Принтер этикеток на воротах приёмки, который только печатает коды, но сам складские операции не сканирует</t>
+          <t xml:space="preserve">Принтер на воротах приёмки: печатает наклейки, но сам штрихкоды с паллет не считывает                    </t>
         </is>
       </c>
       <c r="E31" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Модуль расчёта зарплаты кладовщиков в ERP без функций сканирования штрих- и QR-кодов на складе           </t>
+          <t xml:space="preserve">Программа расчёта зарплаты кладовщиков, без сканера штрихкода и QR на складе                             </t>
         </is>
       </c>
       <c r="F31" s="23" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="C32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Открытый удалённый доступ ко всем контроллерам линии без пароля ради удобства дежурной смены          </t>
+          <t xml:space="preserve">Пустить всех в контроллеры линии из интернета без пароля, «чтобы смене было удобно»                   </t>
         </is>
       </c>
       <c r="D32" s="20" t="inlineStr">
@@ -1757,12 +1757,12 @@
       </c>
       <c r="E32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Хранение единственной копии SCADA на диске оператора без резервирования и контроля сетевого периметра </t>
+          <t xml:space="preserve">Держать единственную копию программы линии на одном компьютере, без запасной копии и защиты сети      </t>
         </is>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Общая учётная запись «оператор» во всех системах без разграничения прав, экранов и резервных копий    </t>
+          <t xml:space="preserve">Один общий логин «оператор» на все компьютеры, без разных прав и без запасных копий                   </t>
         </is>
       </c>
       <c r="G32" s="21" t="n">
@@ -1780,27 +1780,27 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>Почему пиломатериал перед сборкой каркаса поддона пропускают через сушильную камеру?</t>
+          <t>Зачем доски перед сборкой поддона сушат в камере?</t>
         </is>
       </c>
       <c r="C33" s="25" t="inlineStr">
         <is>
-          <t>Чтобы стабилизировать геометрию досок, снизить риск трещин, плесени и ослабления крепежа в эксплуатации</t>
+          <t>Чтобы доски не повело, не пошли трещины и плесень, и гвозди потом не разболтались</t>
         </is>
       </c>
       <c r="D33" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы сырые доски стали тяжелее и промышленный манипулятор надёжнее удерживал заготовку в захвате      </t>
+          <t xml:space="preserve">Чтобы мокрые доски стали тяжелее и роботу было проще их держать в захвате        </t>
         </is>
       </c>
       <c r="E33" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы клеймо ISPM-15 само проявилось на влажной поверхности без отдельной маркировочной станции        </t>
+          <t xml:space="preserve">Чтобы клеймо само проявилось на мокрой доске, без отдельного станка маркировки   </t>
         </is>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы конвейер сборки работал медленнее и такт роботизированной ячейки искусственно удлинился          </t>
+          <t xml:space="preserve">Чтобы конвейер специально ехал медленнее и сборка занимала больше времени        </t>
         </is>
       </c>
       <c r="G33" s="26" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="H33" s="25" t="inlineStr">
         <is>
-          <t>Чтобы стабилизировать геометрию досок, снизить риск трещин, плесени и ослабления крепежа в эксплуатации</t>
+          <t>Чтобы доски не повело, не пошли трещины и плесень, и гвозди потом не разболтались</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Q30 correct: kiln disinfection for food pallets
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -1785,22 +1785,22 @@
       </c>
       <c r="C33" s="25" t="inlineStr">
         <is>
-          <t>Чтобы доски не повело, не пошли трещины и плесень, и гвозди потом не разболтались</t>
+          <t>Чтобы продезинфицировать доски: поддон потом могут поставить под пищевую продукцию</t>
         </is>
       </c>
       <c r="D33" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы мокрые доски стали тяжелее и роботу было проще их держать в захвате        </t>
+          <t xml:space="preserve">Чтобы доски не повело, не пошли трещины, и гвозди потом не разболтались           </t>
         </is>
       </c>
       <c r="E33" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы клеймо само проявилось на мокрой доске, без отдельного станка маркировки   </t>
+          <t xml:space="preserve">Чтобы клеймо само проявилось на мокрой доске, без отдельного станка маркировки    </t>
         </is>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы конвейер специально ехал медленнее и сборка занимала больше времени        </t>
+          <t xml:space="preserve">Чтобы мокрые доски стали тяжелее и роботу было проще держать их в захвате         </t>
         </is>
       </c>
       <c r="G33" s="26" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="H33" s="25" t="inlineStr">
         <is>
-          <t>Чтобы доски не повело, не пошли трещины и плесень, и гвозди потом не разболтались</t>
+          <t>Чтобы продезинфицировать доски: поддон потом могут поставить под пищевую продукцию</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace Q29 IT-contour with plant network isolation
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -180,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -239,6 +239,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1740,37 +1743,37 @@
       <c r="A32" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="20" t="inlineStr">
-        <is>
-          <t>Какой набор мер соответствует защите промышленного IT-контура в модуле?</t>
+      <c r="B32" s="25" t="inlineStr">
+        <is>
+          <t>Зачем контроллеры и компьютеры линии отделяют от обычного интернета и ставят пароли?</t>
         </is>
       </c>
       <c r="C32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Пустить всех в контроллеры линии из интернета без пароля, «чтобы смене было удобно»                   </t>
-        </is>
-      </c>
-      <c r="D32" s="20" t="inlineStr">
-        <is>
-          <t>Мониторинг сетевого трафика, межсетевые экраны и антивирусы, резервное копирование, обучение персонала</t>
+          <t>Чтобы датчики сушилки передавали влажность досок без проводов и без участия оператора</t>
+        </is>
+      </c>
+      <c r="D32" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Чтобы чужие не остановили цех и не подменили программу сборки поддонов               </t>
         </is>
       </c>
       <c r="E32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Держать единственную копию программы линии на одном компьютере, без запасной копии и защиты сети      </t>
+          <t xml:space="preserve">Чтобы пульт робота сам считал зарплату смены и прибыль завода                        </t>
         </is>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Один общий логин «оператор» на все компьютеры, без разных прав и без запасных копий                   </t>
-        </is>
-      </c>
-      <c r="G32" s="21" t="n">
+          <t xml:space="preserve">Чтобы складская программа сама печатала этикетки без сканера и без кладовщика        </t>
+        </is>
+      </c>
+      <c r="G32" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="H32" s="20" t="inlineStr">
-        <is>
-          <t>Мониторинг сетевого трафика, межсетевые экраны и антивирусы, резервное копирование, обучение персонала</t>
+      <c r="H32" s="25" t="inlineStr">
+        <is>
+          <t>Чтобы чужие не остановили цех и не подменили программу сборки поддонов</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Q29 rewritten for pallet assembly module
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -1745,27 +1745,27 @@
       </c>
       <c r="B32" s="25" t="inlineStr">
         <is>
-          <t>Зачем контроллеры и компьютеры линии отделяют от обычного интернета и ставят пароли?</t>
+          <t>Что делает промышленный робот на участке сборки поддона?</t>
         </is>
       </c>
       <c r="C32" s="25" t="inlineStr">
         <is>
-          <t>Чтобы датчики сушилки передавали влажность досок без проводов и без участия оператора</t>
+          <t>Сушит сырые доски в камере, чтобы поддон потом можно было ставить под продукты</t>
         </is>
       </c>
       <c r="D32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы чужие не остановили цех и не подменили программу сборки поддонов               </t>
+          <t>Берёт доску, кладёт её на своё место в каркасе, дальше линия крепит соединение</t>
         </is>
       </c>
       <c r="E32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы пульт робота сам считал зарплату смены и прибыль завода                        </t>
+          <t xml:space="preserve">Ставит клеймо на уже готовую пачку на складе, без участия в сборке каркаса    </t>
         </is>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чтобы складская программа сама печатала этикетки без сканера и без кладовщика        </t>
+          <t xml:space="preserve">Считает зарплату смены и прибыль завода вместо укладки досок на каркас        </t>
         </is>
       </c>
       <c r="G32" s="27" t="n">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="H32" s="25" t="inlineStr">
         <is>
-          <t>Чтобы чужие не остановили цех и не подменили программу сборки поддонов</t>
+          <t>Берёт доску, кладёт её на своё место в каркасе, дальше линия крепит соединение</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rephrase Q29 assembly: where robot places the board
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -1745,27 +1745,27 @@
       </c>
       <c r="B32" s="25" t="inlineStr">
         <is>
-          <t>Что делает промышленный робот на участке сборки поддона?</t>
+          <t>Куда робот должен положить доску после захвата на участке сборки поддона?</t>
         </is>
       </c>
       <c r="C32" s="25" t="inlineStr">
         <is>
-          <t>Сушит сырые доски в камере, чтобы поддон потом можно было ставить под продукты</t>
+          <t xml:space="preserve">Обратно в сушильную камеру, чтобы доска ещё раз прогрелась перед крепежом     </t>
         </is>
       </c>
       <c r="D32" s="25" t="inlineStr">
         <is>
-          <t>Берёт доску, кладёт её на своё место в каркасе, дальше линия крепит соединение</t>
+          <t>На своё место в каркасе на позиции сборки, после этого линия крепит соединение</t>
         </is>
       </c>
       <c r="E32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ставит клеймо на уже готовую пачку на складе, без участия в сборке каркаса    </t>
+          <t xml:space="preserve">Сразу на склад готовой продукции, минуя сборку каркаса и крепёж               </t>
         </is>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Считает зарплату смены и прибыль завода вместо укладки досок на каркас        </t>
+          <t xml:space="preserve">В тару с браком рядом с линией, без укладки в каркас поддона                  </t>
         </is>
       </c>
       <c r="G32" s="27" t="n">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="H32" s="25" t="inlineStr">
         <is>
-          <t>Берёт доску, кладёт её на своё место в каркасе, дальше линия крепит соединение</t>
+          <t>На своё место в каркасе на позиции сборки, после этого линия крепит соединение</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Q29: SOP abbreviation with equal-length lookalike answers
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -1745,27 +1745,27 @@
       </c>
       <c r="B32" s="25" t="inlineStr">
         <is>
-          <t>Куда робот должен положить доску после захвата на участке сборки поддона?</t>
+          <t>Как расшифровывается аббревиатура СОП?</t>
         </is>
       </c>
       <c r="C32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Обратно в сушильную камеру, чтобы доска ещё раз прогрелась перед крепежом     </t>
+          <t>Сквозная организационная процедура</t>
         </is>
       </c>
       <c r="D32" s="25" t="inlineStr">
         <is>
-          <t>На своё место в каркасе на позиции сборки, после этого линия крепит соединение</t>
+          <t>Стандартная операционная процедура</t>
         </is>
       </c>
       <c r="E32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сразу на склад готовой продукции, минуя сборку каркаса и крепёж               </t>
+          <t>Специальная операционная программа</t>
         </is>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">В тару с браком рядом с линией, без укладки в каркас поддона                  </t>
+          <t xml:space="preserve">Стандартный операционный протокол </t>
         </is>
       </c>
       <c r="G32" s="27" t="n">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="H32" s="25" t="inlineStr">
         <is>
-          <t>На своё место в каркасе на позиции сборки, после этого линия крепит соединение</t>
+          <t>Стандартная операционная процедура</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: answers without без/только
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Общий тест 30" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,95 +13,38 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Общий тест 30'!$A$3:$H$33</definedName>
   </definedNames>
-  <calcPr calcId="162913" fullCalcOnLoad="1" refMode="R1C1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color rgb="FF0A2F5C"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color rgb="FF0A2F5C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="134"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FF0A2F5C"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <i val="1"/>
-      <color rgb="FF5A6F88"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF006100"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -109,47 +53,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0A2F5C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F7EF"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FF1457A8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5F8FC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F7EF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5F8FC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -163,89 +72,43 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD0D7E2"/>
+        <color rgb="FFB8C9DE"/>
       </left>
       <right style="thin">
-        <color rgb="FFD0D7E2"/>
+        <color rgb="FFB8C9DE"/>
       </right>
       <top style="thin">
-        <color rgb="FFD0D7E2"/>
+        <color rgb="FFB8C9DE"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD0D7E2"/>
+        <color rgb="FFB8C9DE"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -608,1208 +471,1203 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" style="16" min="1" max="1"/>
-    <col width="42" customWidth="1" style="16" min="2" max="2"/>
-    <col width="32" customWidth="1" style="16" min="3" max="6"/>
-    <col width="12" customWidth="1" style="16" min="7" max="7"/>
-    <col width="32" customWidth="1" style="16" min="8" max="8"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.4" customHeight="1" s="16">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Общий тест ОПП — 30 вопросов </t>
-        </is>
-      </c>
-      <c r="K1" s="24" t="inlineStr">
-        <is>
-          <t>Зелёным — исправленные ответы (проще, без научных терминов)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="13" t="n"/>
-    </row>
-    <row r="3" ht="32.1" customHeight="1" s="16">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Общий тест ОПП — 30 вопросов (варианты равной длины, без «без/только»)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Вопрос</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Вариант A</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Вариант B</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Вариант C</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Вариант D</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Правильный (1=A,2=B,3=C,4=D)</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Текст правильного ответа</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A4" s="6" t="n">
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>В концепции ОПП подготовка кадров Индустрии 4.0 достигается прежде всего за счёт чего?</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Совмещения учебной программы с работой на реальной роботизированной линии и цифровых системах предприятия         </t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Максимального наращивания выпуска экспортных поддонов при полном исключении студентов из производственного контура</t>
         </is>
       </c>
-      <c r="E4" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Проведения только лекций про умный завод без работы студентов на настоящей линии                                  </t>
-        </is>
-      </c>
-      <c r="F4" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Организации только складского хранения готовой тары без допуска обучающихся к действующему оборудованию цеха      </t>
-        </is>
-      </c>
-      <c r="G4" s="21" t="n">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проведения лекционного курса по Индустрии 4.0 вместо практики студентов на действующей линии цеха                 </t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Организации складского хранения готовой тары и запрета обучающимся подходить к оборудованию цеха                  </t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="20" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Совмещения учебной программы с работой на реальной роботизированной линии и цифровых системах предприятия</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A5" s="22" t="n">
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Если выстроить участки ОПП в порядке движения сырья к готовому поддону, какой этап окажется первым?</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Участок сборки, на котором промышленные манипуляторы сразу формируют каркас поддона из уже подготовленных деталей  </t>
-        </is>
-      </c>
-      <c r="D5" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Участок расштабелирования и первичной подготовки пиломатериала перед его направлением в сушильную камеру           </t>
-        </is>
-      </c>
-      <c r="E5" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Линия снятия фасок и нанесения маркировки на уже собранный поддон непосредственно перед отгрузкой клиенту          </t>
-        </is>
-      </c>
-      <c r="F5" s="23" t="inlineStr">
-        <is>
-          <t>Склад готовой продукции, с которого готовая тара без дополнительных операций сразу отправляется конечному заказчику</t>
-        </is>
-      </c>
-      <c r="G5" s="21" t="n">
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Участок сборки, на котором промышленные манипуляторы сразу формируют каркас поддона из уже подготовленных деталей</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Участок расштабелирования и первичной подготовки пиломатериала перед его направлением в сушильную камеру         </t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Линия снятия фасок и нанесения маркировки на уже собранный поддон непосредственно перед отгрузкой клиенту        </t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Склад готовой продукции, с которого готовая тара сразу уходит заказчику, минуя сушку и сборку                    </t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="23" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Участок расштабелирования и первичной подготовки пиломатериала перед его направлением в сушильную камеру</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A6" s="6" t="n">
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Первый промышленный робот Unimate был внедрён на каком предприятии и в каком году?</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">На предприятии KUKA в составе линии опытного производства поддонов в 2010 году                             </t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">На заводе Ford при запуске конвейерной сборки Model T в 1913 году                                          </t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">На заводе General Motors в США в 1961 году как первый промышленный робот                                   </t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>На площадке Siemens в цехе станков с ЧПУ в тысяча девятьсот девяносто пятом году в рамках пилотного проекта</t>
         </is>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>На заводе General Motors в США в 1961 году как первый промышленный робот</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A7" s="22" t="n">
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>На монотонных и опасных операциях робот часто экономически выгоднее человека. Какой аргумент из перечисленных основной?</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Робот всегда обходится предприятию дешевле любого ручного инструмента и не требует энергоснабжения линии</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Роботу не нужны прикладная программа, шкаф управления и регулярное техническое обслуживание привода осей</t>
         </is>
       </c>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Робот самостоятельно заменяет ERP-систему и принимает все управленческие решения без участия инженеров  </t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Робот самостоятельно заменяет ERP-систему и принимает все управленческие решения вместо инженеров       </t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Исключается человеческий фактор, выше стабильность цикла, допускается длительная работа в опасной среде </t>
         </is>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="23" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Исключается человеческий фактор, выше стабильность цикла, допускается длительная работа в опасной среде</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A8" s="6" t="n">
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Ключевое отличие коллаборативного робота (кобота) от классического промышленного робота:</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>Полное отсутствие управляемых осей и серводвигателей в конструкции, из‑за чего кобот движется только вручную</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Возможность эксплуатации исключительно вне атмосферы Земли и в условиях глубокого космического вакуума      </t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Допуск к совместной работе с человеком в одном пространстве без обязательного полного ограждения ячейки     </t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Строгий запрет находиться в зоне конвейера и выполнять любые операции рядом с движущимся грузом на линии    </t>
-        </is>
-      </c>
-      <c r="G8" s="21" t="n">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Полное отсутствие управляемых осей и серводвигателей в конструкции, из‑за чего кобот движется вручную   </t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Возможность эксплуатации исключительно вне атмосферы Земли и в условиях глубокого космического вакуума  </t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Допуск к совместной работе с человеком в одном пространстве, полное ограждение ячейки не обязательно    </t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Строгий запрет находиться в зоне конвейера и выполнять любые операции рядом с движущимся грузом на линии</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="20" t="inlineStr">
-        <is>
-          <t>Допуск к совместной работе с человеком в одном пространстве без обязательного полного ограждения ячейки</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A9" s="22" t="n">
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Допуск к совместной работе с человеком в одном пространстве, полное ограждение ячейки не обязательно</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Для чего нужен пульт SmartPAD?</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Программирования траекторий, запуска и остановки прикладных программ промышленного робота на линии       </t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Управления температурными и влажностными режимами сушильной камеры пиломатериала на участке подготовки   </t>
         </is>
       </c>
-      <c r="E9" s="23" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Печати сертификатов фитосанитарного контроля и этикеток на готовую тару перед отгрузкой со склада        </t>
         </is>
       </c>
-      <c r="F9" s="23" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Автоматического формирования полного отчёта о прибылях и убытках предприятия за выбранный отчётный период</t>
         </is>
       </c>
-      <c r="G9" s="21" t="n">
+      <c r="G9" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="23" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Программирования траекторий, запуска и остановки прикладных программ промышленного робота на линии</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A10" s="6" t="n">
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Зачем в приводе оси промышленного робота ставят редуктор, если сервомотор и так вращается?</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Редуктор охлаждает процессор пульта SmartPAD и снижает нагрев электроники шкафа управления ячейки            </t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Мотор даёт высокие обороты при малом моменте; редуктор снижает скорость и увеличивает момент на выходном валу</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Редуктор хранит пользовательские системы координат World и TCP и подменяет собой память контроллера робота   </t>
-        </is>
-      </c>
-      <c r="F10" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Редуктор полностью заменяет промышленную сеть Profinet и обеспечивает обмен данными между всеми датчиками    </t>
-        </is>
-      </c>
-      <c r="G10" s="21" t="n">
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Редуктор охлаждает процессор пульта SmartPAD и снижает нагрев электроники шкафа управления ячейки                     </t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Мотор даёт высокие обороты при малом моменте; редуктор снижает скорость и увеличивает крутящий момент на выходном валу</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Редуктор хранит пользовательские системы координат World и TCP и подменяет собой память контроллера робота            </t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Редуктор полностью заменяет промышленную сеть Profinet и обеспечивает обмен данными между всеми датчиками             </t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>Мотор даёт высокие обороты при малом моменте; редуктор снижает скорость и увеличивает момент на выходном валу</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A11" s="22" t="n">
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Мотор даёт высокие обороты при малом моменте; редуктор снижает скорость и увеличивает крутящий момент на выходном валу</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Сколько осей (степеней свободы) у промышленного робота в материале модуля?</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Пять  </t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Четыре</t>
         </is>
       </c>
-      <c r="E11" s="23" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Семь  </t>
         </is>
       </c>
-      <c r="F11" s="23" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Шесть </t>
         </is>
       </c>
-      <c r="G11" s="21" t="n">
+      <c r="G11" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="H11" s="23" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Шесть</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A12" s="6" t="n">
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Система координат World у промышленного робота — это:</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Подвижная система отсчёта, жёстко «пришитая» к фланцу инструмента и смещающаяся вместе с каждым движением </t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Неподвижная система отсчёта, связанная с основанием робота и не меняющаяся при движении манипулятора      </t>
         </is>
       </c>
-      <c r="E12" s="20" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Таблица производственных заказов в 1С:ERP, в которой фиксируются позиции и сроки выпуска готовой продукции</t>
         </is>
       </c>
-      <c r="F12" s="20" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Схема маршрута учебной экскурсии по цеху с указанием точек безопасного наблюдения за работой линии        </t>
         </is>
       </c>
-      <c r="G12" s="21" t="n">
+      <c r="G12" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="20" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Неподвижная система отсчёта, связанная с основанием робота и не меняющаяся при движении манипулятора</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A13" s="22" t="n">
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Столкновение манипулятора или грубая ошибка в программе чаще всего приводит к:</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
-        <is>
-          <t>Автоматическому увеличению паспортной грузоподъёмности робота без какого‑либо технического обслуживания</t>
-        </is>
-      </c>
-      <c r="D13" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Самопроизвольному переходу робота в режим кобота с отключением всех защитных ограждений ячейки         </t>
-        </is>
-      </c>
-      <c r="E13" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Рискам повреждения механики и электрики, а также возможной потере текущей калибровки осей манипулятора </t>
-        </is>
-      </c>
-      <c r="F13" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Автоматическому обновлению справочников ERP и пересчёту всех складских остатков без участия оператора  </t>
-        </is>
-      </c>
-      <c r="G13" s="21" t="n">
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Автоматическому увеличению паспортной грузоподъёмности робота и отмене технического обслуживания      </t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Самопроизвольному переходу робота в режим кобота с отключением всех защитных ограждений ячейки        </t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Рискам повреждения механики и электрики, а также возможной потере текущей калибровки осей манипулятора</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Автоматическому обновлению справочников ERP и пересчёту всех складских остатков силами самой программы</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="23" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Рискам повреждения механики и электрики, а также возможной потере текущей калибровки осей манипулятора</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A14" s="6" t="n">
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Экономика производства как дисциплина в первую очередь изучает:</t>
         </is>
       </c>
-      <c r="C14" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Как меняются цены акций на бирже, без связи с тем, как в цехе из досок делают поддон               </t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Как магазины ставят ценники, без учёта сколько реально стоят доски, работа и электричество         </t>
-        </is>
-      </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Биржевые котировки и курсы валют, а не превращение ресурсов цеха в готовую продукцию               </t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Методы розничного ценообразования в магазине, а не материальные и трудовые затраты цеха            </t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Экономические отношения в процессе превращения материальных и трудовых ресурсов в готовую продукцию</t>
         </is>
       </c>
-      <c r="F14" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Какие налоги платит регион, без разбора как материалы и труд превращаются в готовый поддон         </t>
-        </is>
-      </c>
-      <c r="G14" s="21" t="n">
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Налоговые режимы региона и льготы, а не преобразование ресурсов в изделие предприятия              </t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="20" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Экономические отношения в процессе превращения материальных и трудовых ресурсов в готовую продукцию</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A15" s="22" t="n">
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>В модуле по экономике производства выделены четыре смысловых блока. Какой набор верный?</t>
         </is>
       </c>
-      <c r="C15" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Реклама, магазины, красивая коробка и телефон горячей линии — без учёта денег и себестоимости    </t>
-        </is>
-      </c>
-      <c r="D15" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства   </t>
-        </is>
-      </c>
-      <c r="E15" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Кредиты банка, курс валюты, страховка груза и таможня — это не те четыре блока из модуля         </t>
-        </is>
-      </c>
-      <c r="F15" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Корпоративы, льготы, каски и премии сотрудникам — без финансового учёта и себестоимости          </t>
-        </is>
-      </c>
-      <c r="G15" s="21" t="n">
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Маркетинг бренда, розничная сеть и упаковка товара вместо финансового учёта и себестоимости         </t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства      </t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Кредитная политика банка, валютный контроль, страхование грузов и таможенное оформление поставок    </t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Корпоративная культура, соцпакет, охрана труда и мотивация персонала вместо финансовых блоков модуля</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H15" s="23" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A16" s="6" t="n">
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Базовый комплект финансовой отчётности предприятия обычно включает:</t>
         </is>
       </c>
-      <c r="C16" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только список станков и сколько они износились — без прибыли, баланса и движения денег               </t>
-        </is>
-      </c>
-      <c r="D16" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только налоговая бумага и выписка из банка — без полного набора главных финансовых отчётов           </t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Отчёт о прибылях и убытках, бухгалтерский баланс и отчёт о движении денежных средств за период       </t>
-        </is>
-      </c>
-      <c r="F16" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только план продаж и рекламный бюджет — без отчёта о прибыли, баланса и движения денег               </t>
-        </is>
-      </c>
-      <c r="G16" s="21" t="n">
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Ведомость амортизации станков и карточки инвентарных объектов вместо баланса и отчёта о прибыли</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Декларация по НДС и выписка расчётного счёта вместо баланса, прибылей и движения денег         </t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Отчёт о прибылях и убытках, бухгалтерский баланс и отчёт о движении денежных средств за период </t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Прогноз продаж маркетинга и план рекламного бюджета вместо основных форм финансовой отчётности </t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H16" s="20" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Отчёт о прибылях и убытках, бухгалтерский баланс и отчёт о движении денежных средств за период</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A17" s="22" t="n">
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Себестоимость единицы продукции — это:</t>
         </is>
       </c>
-      <c r="C17" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Цена, которую продавец взял «с потолка», не считая свои реальные расходы на поддон                 </t>
-        </is>
-      </c>
-      <c r="D17" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только цена досок, без зарплаты, электричества, износа станков и доставки покупателю               </t>
-        </is>
-      </c>
-      <c r="E17" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Выручка за партию, просто делённая на число людей в смене, без подсчёта всех затрат                </t>
-        </is>
-      </c>
-      <c r="F17" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Сумма всех затрат предприятия на изготовление и реализацию одной единицы готовой продукции         </t>
-        </is>
-      </c>
-      <c r="G17" s="21" t="n">
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Рыночная цена, которую отдел продаж выставил по ощущению рынка, минуя расчёт своих затрат             </t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Прямые затраты на пиломатериал, оставляя в стороне труд, энергию, амортизацию и сбыт                  </t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Плановая выручка партии, механически делённая на число рабочих смены, вместо полной калькуляции затрат</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сумма всех затрат предприятия на изготовление и реализацию одной единицы готовой продукции            </t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="H17" s="23" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Сумма всех затрат предприятия на изготовление и реализацию одной единицы готовой продукции</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A18" s="6" t="n">
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Себестоимость напрямую влияет на три управленческих показателя. Какие?</t>
         </is>
       </c>
-      <c r="C18" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только сколько чиновников в офисе, без цены поддона, конкурентов и прибыли завода                </t>
-        </is>
-      </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Цену предложения на рынке, конкурентоспособность продукции и итоговую прибыльность бизнеса       </t>
-        </is>
-      </c>
-      <c r="E18" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только график ремонта линии, без влияния на цену, конкуренцию и прибыль                          </t>
-        </is>
-      </c>
-      <c r="F18" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только как часто люди увольняются, без связи с ценой поддона и прибылью завода                   </t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="n">
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Численность административного персонала, штатное расписание и график отпусков офиса       </t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Цену предложения на рынке, конкурентоспособность продукции и итоговую прибыльность бизнеса</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">График плановых ремонтов линии, перечень запчастей и даты остановов оборудования          </t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Внутренний индекс текучести кадров, причины увольнений и план найма на квартал            </t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H18" s="20" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Цену предложения на рынке, конкурентоспособность продукции и итоговую прибыльность бизнеса</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A19" s="22" t="n">
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Бюджет на предприятии — это прежде всего:</t>
         </is>
       </c>
-      <c r="C19" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Сколько денег уже прошло через кассу вчера, без плана на месяц, квартал или год             </t>
-        </is>
-      </c>
-      <c r="D19" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Список уже оплаченных счетов поставщикам, без плана доходов и расходов на период            </t>
-        </is>
-      </c>
-      <c r="E19" s="23" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Фактический отчёт кассы за прошедшие сутки и уже состоявшиеся платежи смены                 </t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Реестр уже оплаченных счетов поставщикам и закрытых накладных прошлого месяца               </t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Плановый документ доходов и расходов на выбранный период: месяц, квартал или календарный год</t>
         </is>
       </c>
-      <c r="F19" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Журнал уже сделанных проводок за месяц, без заранее утверждённого плана трат и доходов      </t>
-        </is>
-      </c>
-      <c r="G19" s="21" t="n">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Журнал закрытых бухгалтерских проводок месяца и архив уже сделанных операций                </t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H19" s="23" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Плановый документ доходов и расходов на выбранный период: месяц, квартал или календарный год</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A20" s="6" t="n">
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Под масштабированием в контексте производства понимают:</t>
         </is>
       </c>
-      <c r="C20" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Оставить в продаже только один вид поддона, не увеличивая выпуск и не снижая затраты на штуку       </t>
-        </is>
-      </c>
-      <c r="D20" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Заморозить вложения и часть цеха остановить, чтобы выпускать меньше, а не больше                    </t>
-        </is>
-      </c>
-      <c r="E20" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Набрать только офисных сотрудников, не увеличивая выпуск поддонов и не снижая затраты на штуку      </t>
-        </is>
-      </c>
-      <c r="F20" s="20" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сокращение ассортимента до одной позиции и консервацию части действующих мощностей цеха             </t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Заморозка инвестиций и консервация части мощностей ради снижения, а не роста объёма выпуска         </t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Увеличение офисного штата управляющей компании и рост числа кабинетов администрации                 </t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Рост объёма выпуска или расширение бизнеса ради повышения эффективности и снижения удельных издержек</t>
         </is>
       </c>
-      <c r="G20" s="21" t="n">
+      <c r="G20" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H20" s="20" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Рост объёма выпуска или расширение бизнеса ради повышения эффективности и снижения удельных издержек</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A21" s="22" t="n">
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Вертикальное масштабирование отличается тем, что это:</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Рост «вглубь» цепочки стоимости — контроль поставок сырья и/или выход ближе к конечному потребителю</t>
         </is>
       </c>
-      <c r="D21" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Поставить рядом ещё такие же линии сборки, не заходя в сырьё и не ближе к покупателю               </t>
-        </is>
-      </c>
-      <c r="E21" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Начать выпускать совсем другие товары под тем же названием, не контролируя доски и сбыт            </t>
-        </is>
-      </c>
-      <c r="F21" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Просто увеличить штат офиса, не меняя, кто поставляет доски и кто покупает поддоны                 </t>
-        </is>
-      </c>
-      <c r="G21" s="21" t="n">
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Горизонтальный рост числа однотипных линий того же передела, сырьё и сбыт остаются как были        </t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Концентрический выпуск непрофильных изделий под брендом, сырьё и каналы сбыта остаются чужими      </t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Организационное увеличение штата администрации, цепочка стоимости и близость к клиенту прежние     </t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="23" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>Рост «вглубь» цепочки стоимости — контроль поставок сырья и/или выход ближе к конечному потребителю</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A22" s="6" t="n">
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Инвестиции в производство — это:</t>
         </is>
       </c>
-      <c r="C22" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Обычные счета за свет и расходники, от которых цех не становится больше и поддон не лучше       </t>
-        </is>
-      </c>
-      <c r="D22" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Оплата старого брака, без плана делать больше, качественнее и конкурентоспособнее               </t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Вложения капитала с целью роста объёма выпуска, качества продукции и конкурентоспособности      </t>
-        </is>
-      </c>
-      <c r="F22" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Возврат старого кредита банку, без новых станков и без улучшения поддона                        </t>
-        </is>
-      </c>
-      <c r="G22" s="21" t="n">
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Текущие платежи за энергию и расходники, мощности и качество изделия остаются на прежнем уровне</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Компенсация брака прошлых периодов, выпуск, качество и доля рынка остаются как были            </t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вложения капитала с целью роста объёма выпуска, качества продукции и конкурентоспособности     </t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Возврат ранее взятого кредита банку при прежних мощностях и прежней конкурентоспособности      </t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H22" s="20" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Вложения капитала с целью роста объёма выпуска, качества продукции и конкурентоспособности</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A23" s="22" t="n">
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Какие четыре вида инвестиций названы в учебном модуле?</t>
         </is>
       </c>
-      <c r="C23" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Прямые, косвенные, накладные и торговые затраты в расчёте цены одного поддона               </t>
-        </is>
-      </c>
-      <c r="D23" s="23" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Прямые, косвенные, накладные и коммерческие затраты в калькуляции единицы готовой продукции </t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Капитальные, инновационные, операционные и финансовые вложения в развитие предприятия       </t>
         </is>
       </c>
-      <c r="E23" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Долги на месяц, на год, на много лет и без срока — это про долги, а не про виды вложений    </t>
-        </is>
-      </c>
-      <c r="F23" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Затраты постоянные, переменные и смешанные — это про расходы, а не про четыре вида вложений </t>
-        </is>
-      </c>
-      <c r="G23" s="21" t="n">
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Краткосрочные, среднесрочные, долгосрочные и бессрочные обязательства в структуре баланса   </t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Постоянные, переменные, смешанные и маржинальные издержки в управленческом учёте предприятия</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="23" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Капитальные, инновационные, операционные и финансовые вложения в развитие предприятия</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A24" s="6" t="n">
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>В чём принципиальная разница цифровизации и автоматизации?</t>
         </is>
       </c>
-      <c r="C24" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Цифровизация якобы ставит роботов вместо людей, а автоматизация только сканирует бумажки              </t>
-        </is>
-      </c>
-      <c r="D24" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Автоматизация якобы переводит всё в цифру, а цифровизация — это просто купить ещё датчики             </t>
-        </is>
-      </c>
-      <c r="E24" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Оба слова якобы значат только «купили сервер», без изменений в цехе и в управлении                    </t>
-        </is>
-      </c>
-      <c r="F24" s="20" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Цифровизация заменяет людей машинами, а автоматизация хранит сканы бумажных документов                </t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Автоматизация переводит процессы в данные, а цифровизация сводится к закупке дополнительных датчиков  </t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оба термина означают установку серверов в серверной, цеховые и управленческие процессы прежние        </t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Цифровизация переводит данные и процессы в цифровую форму; автоматизация замещает ручной труд машинами</t>
         </is>
       </c>
-      <c r="G24" s="21" t="n">
+      <c r="G24" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H24" s="20" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Цифровизация переводит данные и процессы в цифровую форму; автоматизация замещает ручной труд машинами</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A25" s="22" t="n">
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Индустрию 1.0 связывают с:</t>
         </is>
       </c>
-      <c r="C25" s="23" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Массовым внедрением искусственного интеллекта на полевом уровне управления оборудованием цеха   </t>
         </is>
       </c>
-      <c r="D25" s="23" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Появлением электрических конвейеров Форда и началом массового поточного производства автомобилей</t>
         </is>
       </c>
-      <c r="E25" s="23" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Концом XVIII века и паровой машиной — переходом от преобладающего ручного труда к машинному     </t>
         </is>
       </c>
-      <c r="F25" s="23" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Внедрением платформы 1С:ERP на российских предприятиях как символом цифровой трансформации      </t>
         </is>
       </c>
-      <c r="G25" s="21" t="n">
+      <c r="G25" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="23" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>Концом XVIII века и паровой машиной — переходом от преобладающего ручного труда к машинному</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A26" s="6" t="n">
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Характерный признак Индустрии 4.0:</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Полный отказ от датчиков и программируемых контроллеров на всех уровнях управления линией                                     </t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Возврат производства исключительно к паровым приводам без использования электрических сервомоторов                            </t>
-        </is>
-      </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Возврат производства к паровым приводам и отказ от электрических сервомоторов на линии                                        </t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Строгий запрет обмена данными между соседними производственными участками внутри одного цеха                                  </t>
         </is>
       </c>
-      <c r="F26" s="20" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Интеграция цифровых и физических систем, при которой оборудование, датчики, ПО и люди обмениваются данными в реальном времени.</t>
         </is>
       </c>
-      <c r="G26" s="21" t="n">
+      <c r="G26" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H26" s="20" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Интеграция цифровых и физических систем, при которой оборудование, датчики, ПО и люди обмениваются данными в реальном времени.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A27" s="22" t="n">
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="23" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>ERP-система на предприятии — это:</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только видеокамера внутри сушильной камеры, передающая изображение оператору смены на монитор </t>
-        </is>
-      </c>
-      <c r="D27" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только teach-пульт SmartPAD, с помощью которого настраивают траектории движения манипулятора  </t>
-        </is>
-      </c>
-      <c r="E27" s="23" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Видеокамера внутри сушильной камеры, передающая изображение оператору смены на монитор        </t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Система, с помощью которой настраивают траектории движения манипулятора                       </t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Единая цифровая платформа, объединяющая производство, склад, продажи, финансы и учёт персонала</t>
         </is>
       </c>
-      <c r="F27" s="23" t="inlineStr">
-        <is>
-          <t>Только механический редуктор шестой оси робота, снижающий обороты сервомотора на выходном валу</t>
-        </is>
-      </c>
-      <c r="G27" s="21" t="n">
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Механический редуктор шестой оси робота, снижающий обороты сервомотора на выходном валу       </t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="23" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Единая цифровая платформа, объединяющая производство, склад, продажи, финансы и учёт персонала</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A28" s="6" t="n">
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Почему PLC образно называют «рефлексами» производства?</t>
         </is>
       </c>
-      <c r="C28" s="20" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Контроллер в реальном времени обрабатывает сигналы датчиков и выдаёт быстрые локальные команды приводам</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">PLC самостоятельно формирует полный пакет годовой финансовой отчётности для акционеров предприятия     </t>
         </is>
       </c>
-      <c r="E28" s="20" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">PLC хранит кадровые резюме сотрудников и заменяет собой систему управления персоналом на заводе        </t>
         </is>
       </c>
-      <c r="F28" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLC выполняет функции складского перегрузчика и перемещает паллеты без участия складской техники       </t>
-        </is>
-      </c>
-      <c r="G28" s="21" t="n">
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLC выполняет функции складского перегрузчика и сам перемещает паллеты вместо складской техники        </t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="20" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Контроллер в реальном времени обрабатывает сигналы датчиков и выдаёт быстрые локальные команды приводам</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A29" s="22" t="n">
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="23" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>MES-система в текущем производстве «знает» прежде всего:</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только актуальный биржевой курс валют, необходимый для расчёта экспортных контрактов предприятия  </t>
-        </is>
-      </c>
-      <c r="D29" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Какой заказ сейчас в работе, фактический выпуск, уровень брака и текущую загрузку оборудования    </t>
-        </is>
-      </c>
-      <c r="E29" s="23" t="inlineStr">
-        <is>
-          <t>Только список экскурсоводов смены и расписание учебных групп, посещающих производственную площадку</t>
-        </is>
-      </c>
-      <c r="F29" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Только заводской цвет корпуса конкретного манипулятора без данных о заказах и производительности  </t>
-        </is>
-      </c>
-      <c r="G29" s="21" t="n">
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Актуальный биржевой курс валют, нужный для расчёта экспортных контрактов предприятия          </t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Какой заказ сейчас в работе, фактический выпуск, уровень брака и текущую загрузку оборудования</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Список экскурсоводов смены и расписание учебных групп, посещающих производственную площадку   </t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Заводской цвет корпуса конкретного манипулятора и каталожный номер корпуса в спецификации     </t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H29" s="23" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>Какой заказ сейчас в работе, фактический выпуск, уровень брака и текущую загрузку оборудования</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A30" s="6" t="n">
+    <row r="30" ht="48" customHeight="1">
+      <c r="A30" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>WMS — это система, которая отвечает за:</t>
         </is>
       </c>
-      <c r="C30" s="20" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Управление осями и скоростями промышленного манипулятора в рамках прикладной программы ячейки</t>
         </is>
       </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Измерение угла поворота ротора сервомотора и передачу этих данных в систему координат World  </t>
         </is>
       </c>
-      <c r="E30" s="20" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Управление складскими процессами предприятия от приёмки товара до комплектации и отгрузки    </t>
         </is>
       </c>
-      <c r="F30" s="20" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Формирование отчёта о движении денежных средств и закрытие финансового периода бухгалтерией  </t>
         </is>
       </c>
-      <c r="G30" s="21" t="n">
+      <c r="G30" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H30" s="20" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>Управление складскими процессами предприятия от приёмки товара до комплектации и отгрузки</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A31" s="22" t="n">
+    <row r="31" ht="48" customHeight="1">
+      <c r="A31" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>ТСД в контуре WMS — это:</t>
         </is>
       </c>
-      <c r="C31" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Большой компьютер склада, где лежат списки товара и остатки, но им не сканируют коробки в руках          </t>
-        </is>
-      </c>
-      <c r="D31" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Принтер на воротах приёмки: печатает наклейки, но сам штрихкоды с паллет не считывает                    </t>
-        </is>
-      </c>
-      <c r="E31" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Программа расчёта зарплаты кладовщиков, без сканера штрихкода и QR на складе                             </t>
-        </is>
-      </c>
-      <c r="F31" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Терминал сбора данных: мобильное устройство со сканером штрих‑ или QR‑кодов для складских операций       </t>
-        </is>
-      </c>
-      <c r="G31" s="21" t="n">
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стационарный сервер WMS, на котором хранятся складские справочники, остатки и история движений    </t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Принтер этикеток на воротах приёмки, который печатает коды и оставляет сканирование кладовщику    </t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Модуль расчёта зарплаты кладовщиков в ERP вместо сканера штрих- и QR-кодов на складе              </t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Терминал сбора данных: мобильное устройство со сканером штрих‑ или QR‑кодов для складских операций</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="H31" s="23" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Терминал сбора данных: мобильное устройство со сканером штрих‑ или QR‑кодов для складских операций</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A32" s="6" t="n">
+    <row r="32" ht="48" customHeight="1">
+      <c r="A32" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="25" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Как расшифровывается аббревиатура СОП?</t>
         </is>
       </c>
-      <c r="C32" s="25" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Стандартные операционные процедуры</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Специальная операционная программа</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стандартный операционный протокол </t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>Сквозная организационная процедура</t>
         </is>
       </c>
-      <c r="D32" s="25" t="inlineStr">
-        <is>
-          <t>Стандартная операционная процедура</t>
-        </is>
-      </c>
-      <c r="E32" s="25" t="inlineStr">
-        <is>
-          <t>Специальная операционная программа</t>
-        </is>
-      </c>
-      <c r="F32" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Стандартный операционный протокол </t>
-        </is>
-      </c>
-      <c r="G32" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="H32" s="25" t="inlineStr">
-        <is>
-          <t>Стандартная операционная процедура</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="87.90000000000001" customHeight="1" s="16">
-      <c r="A33" s="22" t="n">
+      <c r="G32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Стандартные операционные процедуры</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1">
+      <c r="A33" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="25" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Почему пиломатериал перед сборкой каркаса поддона пропускают через сушильную камеру?</t>
         </is>
       </c>
-      <c r="C33" s="25" t="inlineStr">
-        <is>
-          <t>Чтобы продезинфицировать доски: поддон потом могут поставить под пищевую продукцию</t>
-        </is>
-      </c>
-      <c r="D33" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Чтобы доски не повело, не пошли трещины, и гвозди потом не разболтались           </t>
-        </is>
-      </c>
-      <c r="E33" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Чтобы клеймо само проявилось на мокрой доске, без отдельного станка маркировки    </t>
-        </is>
-      </c>
-      <c r="F33" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Чтобы мокрые доски стали тяжелее и роботу было проще держать их в захвате         </t>
-        </is>
-      </c>
-      <c r="G33" s="26" t="n">
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Чтобы продезинфицировать доски: поддон потом могут поставить под пищевую продукцию               </t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Чтобы сырые доски стали тяжелее и промышленный манипулятор надёжнее удерживал заготовку в захвате</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Чтобы серийный номер сам проявился на влажной поверхности, минуя маркировочную станцию           </t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Чтобы конвейер сборки работал медленнее и такт роботизированной ячейки искусственно удлинился    </t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H33" s="25" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Чтобы продезинфицировать доски: поддон потом могут поставить под пищевую продукцию</t>
         </is>
@@ -1817,8 +1675,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:H33"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1832,426 +1689,426 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C34"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="15.6" customHeight="1" s="16">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ключ (равная длина)</t>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Ключ</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Правильный</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Буква</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" t="n">
         <v>2</v>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" t="n">
         <v>4</v>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" t="n">
         <v>4</v>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" t="n">
         <v>2</v>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" t="n">
         <v>4</v>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" t="n">
         <v>3</v>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" t="n">
         <v>4</v>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" t="n">
         <v>24</v>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" t="n">
         <v>3</v>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
+      <c r="A27" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" t="n">
         <v>1</v>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
+      <c r="A28" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" t="n">
         <v>2</v>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
+      <c r="A29" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B29" t="n">
         <v>3</v>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
+      <c r="A30" t="n">
         <v>28</v>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" t="n">
         <v>4</v>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
+      <c r="A32" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" t="n">
         <v>1</v>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Распределение: A=5, B=8, C=10, D=7</t>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Распределение: A=6, B=7, C=10, D=7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel synced with harder 12/14/21/23/24
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,19 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +70,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5F8FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -105,6 +121,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -475,23 +500,23 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Общий тест ОПП — 30 вопросов (варианты равной длины, без «без/только»)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
+          <t>Общий тест ОПП — 30 вопросов</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>№</t>
@@ -533,7 +558,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="4" ht="52" customHeight="1">
       <c r="A4" s="3" t="n">
         <v>1</v>
       </c>
@@ -571,7 +596,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1">
+    <row r="5" ht="52" customHeight="1">
       <c r="A5" s="5" t="n">
         <v>2</v>
       </c>
@@ -609,7 +634,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="52" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>3</v>
       </c>
@@ -647,7 +672,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="52" customHeight="1">
       <c r="A7" s="5" t="n">
         <v>4</v>
       </c>
@@ -685,7 +710,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="52" customHeight="1">
       <c r="A8" s="3" t="n">
         <v>5</v>
       </c>
@@ -723,7 +748,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="52" customHeight="1">
       <c r="A9" s="5" t="n">
         <v>6</v>
       </c>
@@ -761,7 +786,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
+    <row r="10" ht="52" customHeight="1">
       <c r="A10" s="3" t="n">
         <v>7</v>
       </c>
@@ -799,7 +824,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="52" customHeight="1">
       <c r="A11" s="5" t="n">
         <v>8</v>
       </c>
@@ -837,7 +862,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="52" customHeight="1">
       <c r="A12" s="3" t="n">
         <v>9</v>
       </c>
@@ -875,7 +900,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="52" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>10</v>
       </c>
@@ -913,7 +938,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
+    <row r="14" ht="52" customHeight="1">
       <c r="A14" s="3" t="n">
         <v>11</v>
       </c>
@@ -951,121 +976,121 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="5" t="n">
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>В модуле по экономике производства выделены четыре смысловых блока. Какой набор верный?</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Маркетинг бренда, розничная сеть и упаковка товара вместо финансового учёта и себестоимости         </t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства      </t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Кредитная политика банка, валютный контроль, страхование грузов и таможенное оформление поставок    </t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Корпоративная культура, соцпакет, охрана труда и мотивация персонала вместо финансовых блоков модуля</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n">
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Маркетинг бренда, розничная сеть, дизайн упаковки и программа лояльности клиентов               </t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства  </t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Кредитная политика банка, валютный контроль, страхование грузов и таможенное оформление поставок</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Корпоративная культура, соцпакет, охрана труда и система мотивации персонала                    </t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="3" t="n">
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Базовый комплект финансовой отчётности предприятия обычно включает:</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Ведомость амортизации станков и карточки инвентарных объектов вместо баланса и отчёта о прибыли</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Декларация по НДС и выписка расчётного счёта вместо баланса, прибылей и движения денег         </t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Отчёт о прибылях и убытках, бухгалтерский баланс и отчёт о движении денежных средств за период </t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Прогноз продаж маркетинга и план рекламного бюджета вместо основных форм финансовой отчётности </t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Отчёт о прибылях и убытках, бухгалтерский баланс и отчёт о движении денежных средств за период</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="5" t="n">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>В каком году по задаче генерального директора началась разработка концепта технологичного производства для обучения участников дуальной программы АП?</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>2021 год</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>2020 год</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>2022 год</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>2019 год</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>2019 год</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Себестоимость единицы продукции — это:</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Рыночная цена, которую отдел продаж выставил по ощущению рынка, минуя расчёт своих затрат             </t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Прямые затраты на пиломатериал, оставляя в стороне труд, энергию, амортизацию и сбыт                  </t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Плановая выручка партии, механически делённая на число рабочих смены, вместо полной калькуляции затрат</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Сумма всех затрат предприятия на изготовление и реализацию одной единицы готовой продукции            </t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n">
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Цена, которую отдел продаж согласовал с покупателем на переговорах                        </t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Затраты на пиломатериал по накладной поставщика досок на склад                            </t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выручка за партию, делённая на число рабочих, вышедших в смену                            </t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Сумма всех затрат предприятия на изготовление и реализацию одной единицы готовой продукции</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>Сумма всех затрат предприятия на изготовление и реализацию одной единицы готовой продукции</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1">
+    <row r="18" ht="52" customHeight="1">
       <c r="A18" s="3" t="n">
         <v>15</v>
       </c>
@@ -1103,7 +1128,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
+    <row r="19" ht="52" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>16</v>
       </c>
@@ -1141,7 +1166,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1">
+    <row r="20" ht="52" customHeight="1">
       <c r="A20" s="3" t="n">
         <v>17</v>
       </c>
@@ -1179,7 +1204,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1">
+    <row r="21" ht="52" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>18</v>
       </c>
@@ -1217,7 +1242,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="48" customHeight="1">
+    <row r="22" ht="52" customHeight="1">
       <c r="A22" s="3" t="n">
         <v>19</v>
       </c>
@@ -1255,7 +1280,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="48" customHeight="1">
+    <row r="23" ht="52" customHeight="1">
       <c r="A23" s="5" t="n">
         <v>20</v>
       </c>
@@ -1293,45 +1318,45 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="3" t="n">
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>В чём принципиальная разница цифровизации и автоматизации?</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Цифровизация заменяет людей машинами, а автоматизация хранит сканы бумажных документов                </t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Автоматизация переводит процессы в данные, а цифровизация сводится к закупке дополнительных датчиков  </t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Оба термина означают установку серверов в серверной, цеховые и управленческие процессы прежние        </t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Цифровизация замещает ручной труд машинами, автоматизация переводит данные и процессы в цифровую форму</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Цифровизация касается документов офиса, автоматизация касается роботов и конвейера в цехе             </t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">В модуле это одно и то же: оба слова называют этап внедрения 1С:ERP на предприятии                    </t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Цифровизация переводит данные и процессы в цифровую форму; автоматизация замещает ручной труд машинами</t>
         </is>
       </c>
-      <c r="G24" s="3" t="n">
+      <c r="G24" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>Цифровизация переводит данные и процессы в цифровую форму; автоматизация замещает ручной труд машинами</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1">
+    <row r="25" ht="52" customHeight="1">
       <c r="A25" s="5" t="n">
         <v>22</v>
       </c>
@@ -1369,83 +1394,83 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="48" customHeight="1">
-      <c r="A26" s="3" t="n">
+    <row r="26" ht="52" customHeight="1">
+      <c r="A26" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Характерный признак Индустрии 4.0:</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Полный отказ от датчиков и программируемых контроллеров на всех уровнях управления линией                                     </t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Возврат производства к паровым приводам и отказ от электрических сервомоторов на линии                                        </t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Строгий запрет обмена данными между соседними производственными участками внутри одного цеха                                  </t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Интеграция цифровых и физических систем, при которой оборудование, датчики, ПО и люди обмениваются данными в реальном времени.</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="n">
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Массовое поточное производство на электрическом конвейере с разделением операций                                             </t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Широкое внедрение ЧПУ и программируемых контроллеров как основы автоматизации цеха                                           </t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Паровая машина и переход от ручного труда к машинному на мануфактуре                                                         </t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Интеграция цифровых и физических систем, при которой оборудование, датчики, ПО и люди обмениваются данными в реальном времени</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Интеграция цифровых и физических систем, при которой оборудование, датчики, ПО и люди обмениваются данными в реальном времени.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="48" customHeight="1">
-      <c r="A27" s="5" t="n">
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Интеграция цифровых и физических систем, при которой оборудование, датчики, ПО и люди обмениваются данными в реальном времени</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="52" customHeight="1">
+      <c r="A27" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>ERP-система на предприятии — это:</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Видеокамера внутри сушильной камеры, передающая изображение оператору смены на монитор        </t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Система, с помощью которой настраивают траектории движения манипулятора                       </t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Система оперативного управления цехом: какой заказ в работе, выпуск, брак и загрузка станков  </t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Система управления складом: приёмка, размещение в ячейках, комплектация и отгрузка            </t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>Единая цифровая платформа, объединяющая производство, склад, продажи, финансы и учёт персонала</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Механический редуктор шестой оси робота, снижающий обороты сервомотора на выходном валу       </t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="n">
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Контроллер, который по сигналам датчиков в реальном времени выдаёт команды приводам линии     </t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H27" s="8" t="inlineStr">
         <is>
           <t>Единая цифровая платформа, объединяющая производство, склад, продажи, финансы и учёт персонала</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="48" customHeight="1">
+    <row r="28" ht="52" customHeight="1">
       <c r="A28" s="3" t="n">
         <v>25</v>
       </c>
@@ -1483,7 +1508,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="48" customHeight="1">
+    <row r="29" ht="52" customHeight="1">
       <c r="A29" s="5" t="n">
         <v>26</v>
       </c>
@@ -1521,7 +1546,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="48" customHeight="1">
+    <row r="30" ht="52" customHeight="1">
       <c r="A30" s="3" t="n">
         <v>27</v>
       </c>
@@ -1559,7 +1584,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="48" customHeight="1">
+    <row r="31" ht="52" customHeight="1">
       <c r="A31" s="5" t="n">
         <v>28</v>
       </c>
@@ -1597,7 +1622,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="48" customHeight="1">
+    <row r="32" ht="52" customHeight="1">
       <c r="A32" s="3" t="n">
         <v>29</v>
       </c>
@@ -1635,7 +1660,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="48" customHeight="1">
+    <row r="33" ht="52" customHeight="1">
       <c r="A33" s="5" t="n">
         <v>30</v>
       </c>
@@ -1876,11 +1901,11 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2133,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Распределение: A=6, B=7, C=10, D=7</t>
+          <t>Распределение: A=6, B=7, C=9, D=8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel Q12 production-economics only
</commit_message>
<xml_diff>
--- a/OPP-voprosy-ispravlennye.xlsx
+++ b/OPP-voprosy-ispravlennye.xlsx
@@ -104,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -130,6 +130,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -987,25 +990,25 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Маркетинг бренда, розничная сеть, дизайн упаковки и программа лояльности клиентов               </t>
+          <t xml:space="preserve">Выручка, прибыль, амортизация станков и оборотный капитал предприятия                         </t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства  </t>
+          <t>Финансовый учёт, себестоимость продукции, инвестиции в развитие и масштабирование производства</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Кредитная политика банка, валютный контроль, страхование грузов и таможенное оформление поставок</t>
+          <t xml:space="preserve">Прямые затраты, накладные расходы, фонд оплаты труда и стоимость электроэнергии               </t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Корпоративная культура, соцпакет, охрана труда и система мотивации персонала                    </t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="n">
+          <t xml:space="preserve">Бюджет периода, отчёт о движении денег, бухгалтерский баланс и налоговая декларация           </t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="n">
         <v>2</v>
       </c>
       <c r="H15" s="8" t="inlineStr">

</xml_diff>